<commit_message>
chore: sentiment results 2026-05-03
</commit_message>
<xml_diff>
--- a/results/endesa-sentiment-2026-05-03.xlsx
+++ b/results/endesa-sentiment-2026-05-03.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
   <si>
     <t>Metric</t>
   </si>
@@ -96,6 +96,35 @@
   </si>
   <si>
     <t>Collected At</t>
+  </si>
+  <si>
+    <t>AxVake</t>
+  </si>
+  <si>
+    <t>Cancelamento serviço prosegur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Olá a todos
+Escrevo aqui no ambito de ter uma opinião e possiveis conselhos de como poderei proceder para cancelar da melhor forma o meu serviço da prosegur alarmes. Deixo aqui o contexto total para perceberem:
+Em setembro do ano passado decidi colocar um alarme da prosegur na obra da minha casa uma vez que foram lá roubar-me várias ferramentas. Liguei para o nº geral e apareceram 2 vendedores que me garantiram que era tudo possível e viável, mesmo estando a obra a decorrer obras, que seria su</t>
+  </si>
+  <si>
+    <t>https://www.reddit.com/r/portugal/comments/1sy5gip/cancelamento_servi%C3%A7o_prosegur/</t>
+  </si>
+  <si>
+    <t>portugal</t>
+  </si>
+  <si>
+    <t>2026-04-28T15:55:38.000Z</t>
+  </si>
+  <si>
+    <t>-5.000</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>2026-05-03T17:44:19.030Z</t>
   </si>
   <si>
     <t>Special_Chart2975</t>
@@ -112,9 +141,6 @@
     <t>https://www.reddit.com/r/portugal/comments/1skea7k/endesa_altera%C3%A7%C3%A3o_de_dados_sem_o_meu_conhecimento/</t>
   </si>
   <si>
-    <t>portugal</t>
-  </si>
-  <si>
     <t>2026-04-13T15:30:34.000Z</t>
   </si>
   <si>
@@ -122,35 +148,6 @@
   </si>
   <si>
     <t>No</t>
-  </si>
-  <si>
-    <t>2026-05-03T16:00:40.917Z</t>
-  </si>
-  <si>
-    <t>AxVake</t>
-  </si>
-  <si>
-    <t>Cancelamento serviço prosegur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Olá a todos
-Escrevo aqui no ambito de ter uma opinião e possiveis conselhos de como poderei proceder para cancelar da melhor forma o meu serviço da prosegur alarmes. Deixo aqui o contexto total para perceberem:
-Em setembro do ano passado decidi colocar um alarme da prosegur na obra da minha casa uma vez que foram lá roubar-me várias ferramentas. Liguei para o nº geral e apareceram 2 vendedores que me garantiram que era tudo possível e viável, mesmo estando a obra a decorrer obras, que seria su</t>
-  </si>
-  <si>
-    <t>https://www.reddit.com/r/portugal/comments/1sy5gip/cancelamento_servi%C3%A7o_prosegur/</t>
-  </si>
-  <si>
-    <t>2026-04-28T15:55:38.000Z</t>
-  </si>
-  <si>
-    <t>-5.000</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>2026-05-03T16:00:40.919Z</t>
   </si>
 </sst>
 </file>
@@ -239,13 +236,13 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -768,12 +765,12 @@
         <v>33</v>
       </c>
       <c r="G2" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H2" s="5">
-        <v>5</v>
-      </c>
-      <c r="I2" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" s="7" t="s">
         <v>34</v>
       </c>
       <c r="J2" s="5" t="s">
@@ -784,38 +781,38 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="G3" s="7">
-        <v>2</v>
-      </c>
-      <c r="H3" s="7">
-        <v>20</v>
-      </c>
-      <c r="I3" s="9" t="s">
+      <c r="G3" s="8">
+        <v>1</v>
+      </c>
+      <c r="H3" s="8">
+        <v>5</v>
+      </c>
+      <c r="I3" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="J3" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="K3" s="7" t="s">
-        <v>44</v>
+      <c r="K3" s="8" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>